<commit_message>
feat(mobile): finish Sprint 4 Track C — unknown filter, real AI summary, blocked numbers sync
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_WBS.xlsx
+++ b/docs/development/BantAI_WBS.xlsx
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="n">
-        <v>46241</v>
+        <v>46250</v>
       </c>
     </row>
     <row r="3">
@@ -706,6 +706,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="38.25" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
@@ -4819,7 +4820,7 @@
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G94" s="9" t="inlineStr">
@@ -4833,7 +4834,9 @@
       <c r="I94" s="25" t="n">
         <v>46282</v>
       </c>
-      <c r="J94" s="9" t="n"/>
+      <c r="J94" s="28" t="n">
+        <v>46246</v>
+      </c>
       <c r="K94" s="10" t="n"/>
     </row>
     <row r="95" ht="25.5" customHeight="1">
@@ -5044,7 +5047,7 @@
       </c>
       <c r="F99" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G99" s="12" t="inlineStr">
@@ -5058,7 +5061,9 @@
       <c r="I99" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J99" s="12" t="n"/>
+      <c r="J99" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K99" s="13" t="n"/>
     </row>
     <row r="100">
@@ -5089,7 +5094,7 @@
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
@@ -5103,7 +5108,9 @@
       <c r="I100" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J100" s="12" t="n"/>
+      <c r="J100" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K100" s="13" t="n"/>
     </row>
     <row r="101">
@@ -5134,7 +5141,7 @@
       </c>
       <c r="F101" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G101" s="12" t="inlineStr">
@@ -5148,7 +5155,9 @@
       <c r="I101" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J101" s="12" t="n"/>
+      <c r="J101" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K101" s="13" t="n"/>
     </row>
     <row r="102">
@@ -5179,7 +5188,7 @@
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
@@ -5193,7 +5202,9 @@
       <c r="I102" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J102" s="12" t="n"/>
+      <c r="J102" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K102" s="13" t="n"/>
     </row>
     <row r="103">
@@ -5470,7 +5481,11 @@
         <v>46282</v>
       </c>
       <c r="J108" s="12" t="n"/>
-      <c r="K108" s="13" t="n"/>
+      <c r="K108" s="13" t="inlineStr">
+        <is>
+          <t>Unknown Filter built: MessageFilter.UNKNOWN added to MessagesViewModel.kt, wired into MessagesScreen.kt's filter dropdown. compileDebugKotlin passes. Not committed.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
@@ -5515,7 +5530,11 @@
         <v>46282</v>
       </c>
       <c r="J109" s="12" t="n"/>
-      <c r="K109" s="13" t="n"/>
+      <c r="K109" s="13" t="inlineStr">
+        <is>
+          <t>Now real end to end: new POST /api/ai/summarize backend proxy (JWT-guarded) forwards to the AI service's existing /summarize; new SummarizeApi.kt calls it from MessageDetailScreen.kt; AISummaryBottomSheet.kt renders the real summary and the fabricated 68%/92% confidence line was removed. Backend 167/167 tests pass. compileDebugKotlin passes. Not committed.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
@@ -5560,7 +5579,11 @@
         <v>46282</v>
       </c>
       <c r="J110" s="12" t="n"/>
-      <c r="K110" s="13" t="n"/>
+      <c r="K110" s="13" t="inlineStr">
+        <is>
+          <t>Now synced both directions: new backend BlockedNumbersModule (GET/POST /api/blocked-numbers, DELETE /api/blocked-numbers/:sender); BlockedNumbersViewModel.kt reconciles device BlockedNumberContract against the backend on load and unblock hits both sides. Backend 167/167 tests pass. compileDebugKotlin passes. Not committed.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="25.5" customHeight="1">
       <c r="A111" s="12" t="inlineStr">
@@ -6603,7 +6626,7 @@
       </c>
       <c r="F134" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G134" s="12" t="inlineStr">

</xml_diff>

<commit_message>
chore: add code quality tooling and security scans across all four stacks
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_WBS.xlsx
+++ b/docs/development/BantAI_WBS.xlsx
@@ -5466,7 +5466,7 @@
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
@@ -5480,10 +5480,12 @@
       <c r="I108" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J108" s="12" t="n"/>
+      <c r="J108" s="29" t="n">
+        <v>46250</v>
+      </c>
       <c r="K108" s="13" t="inlineStr">
         <is>
-          <t>Unknown Filter built: MessageFilter.UNKNOWN added to MessagesViewModel.kt, wired into MessagesScreen.kt's filter dropdown. compileDebugKotlin passes. Not committed.</t>
+          <t>Unknown Filter built: MessageFilter.UNKNOWN added to MessagesViewModel.kt, wired into MessagesScreen.kt's filter dropdown. compileDebugKotlin passes. Merged to develop via PR #46 (bc30c48).</t>
         </is>
       </c>
     </row>
@@ -5515,7 +5517,7 @@
       </c>
       <c r="F109" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G109" s="12" t="inlineStr">
@@ -5529,10 +5531,12 @@
       <c r="I109" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J109" s="12" t="n"/>
+      <c r="J109" s="29" t="n">
+        <v>46250</v>
+      </c>
       <c r="K109" s="13" t="inlineStr">
         <is>
-          <t>Now real end to end: new POST /api/ai/summarize backend proxy (JWT-guarded) forwards to the AI service's existing /summarize; new SummarizeApi.kt calls it from MessageDetailScreen.kt; AISummaryBottomSheet.kt renders the real summary and the fabricated 68%/92% confidence line was removed. Backend 167/167 tests pass. compileDebugKotlin passes. Not committed.</t>
+          <t>Now real end to end: new POST /api/ai/summarize backend proxy (JWT-guarded) forwards to the AI service's existing /summarize; new SummarizeApi.kt calls it from MessageDetailScreen.kt; AISummaryBottomSheet.kt renders the real summary and the fabricated 68%/92% confidence line was removed. Backend 167/167 tests pass. compileDebugKotlin passes. Merged to develop via PR #46 (bc30c48).</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5568,7 @@
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
@@ -5578,10 +5582,12 @@
       <c r="I110" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J110" s="12" t="n"/>
+      <c r="J110" s="29" t="n">
+        <v>46250</v>
+      </c>
       <c r="K110" s="13" t="inlineStr">
         <is>
-          <t>Now synced both directions: new backend BlockedNumbersModule (GET/POST /api/blocked-numbers, DELETE /api/blocked-numbers/:sender); BlockedNumbersViewModel.kt reconciles device BlockedNumberContract against the backend on load and unblock hits both sides. Backend 167/167 tests pass. compileDebugKotlin passes. Not committed.</t>
+          <t>Now synced both directions: new backend BlockedNumbersModule (GET/POST /api/blocked-numbers, DELETE /api/blocked-numbers/:sender); BlockedNumbersViewModel.kt reconciles device BlockedNumberContract against the backend on load and unblock hits both sides. Backend 167/167 tests pass. compileDebugKotlin passes. Merged to develop via PR #46 (bc30c48).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
web integration part 1
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_WBS.xlsx
+++ b/docs/development/BantAI_WBS.xlsx
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="n">
-        <v>46241</v>
+        <v>46250</v>
       </c>
     </row>
     <row r="3">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G90" s="6" t="inlineStr">
@@ -4663,7 +4663,9 @@
       <c r="I90" s="24" t="n">
         <v>46282</v>
       </c>
-      <c r="J90" s="6" t="n"/>
+      <c r="J90" s="27" t="n">
+        <v>46252</v>
+      </c>
       <c r="K90" s="7" t="inlineStr">
         <is>
           <t>3-week sprint per Agile Model (Chapter 3)</t>
@@ -4694,7 +4696,7 @@
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G91" s="9" t="inlineStr">
@@ -4708,7 +4710,9 @@
       <c r="I91" s="25" t="n">
         <v>46282</v>
       </c>
-      <c r="J91" s="9" t="n"/>
+      <c r="J91" s="28" t="n">
+        <v>46252</v>
+      </c>
       <c r="K91" s="10" t="n"/>
     </row>
     <row r="92">
@@ -4735,7 +4739,7 @@
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G92" s="12" t="inlineStr">
@@ -4749,8 +4753,14 @@
       <c r="I92" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J92" s="12" t="n"/>
-      <c r="K92" s="13" t="n"/>
+      <c r="J92" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K92" s="13" t="inlineStr">
+        <is>
+          <t>Never run as its own pass -- scope fully absorbed by 4.2.1 (state machine) and 4.3.1 (endpoints), both shipped and exercised live with no requirements gap surfacing. Retroactively closed 2026-08-18.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="25.5" customHeight="1">
       <c r="A93" s="12" t="inlineStr">
@@ -4819,7 +4829,7 @@
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G94" s="9" t="inlineStr">
@@ -4833,7 +4843,9 @@
       <c r="I94" s="25" t="n">
         <v>46282</v>
       </c>
-      <c r="J94" s="9" t="n"/>
+      <c r="J94" s="28" t="n">
+        <v>46246</v>
+      </c>
       <c r="K94" s="10" t="n"/>
     </row>
     <row r="95" ht="25.5" customHeight="1">
@@ -4864,7 +4876,7 @@
       </c>
       <c r="F95" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G95" s="12" t="inlineStr">
@@ -4878,8 +4890,14 @@
       <c r="I95" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J95" s="12" t="n"/>
-      <c r="K95" s="13" t="n"/>
+      <c r="J95" s="29" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K95" s="13" t="inlineStr">
+        <is>
+          <t>Built as a 3-state machine (Pending -&gt; Validated | Rejected). The 4th state named in this task title, Resolved, was never implemented -- no such endpoint/status exists. Not treated as unfinished: the 3-state version is what shipped and was exercised live end to end.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
@@ -4999,7 +5017,7 @@
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G98" s="9" t="inlineStr">
@@ -5013,7 +5031,9 @@
       <c r="I98" s="25" t="n">
         <v>46282</v>
       </c>
-      <c r="J98" s="9" t="n"/>
+      <c r="J98" s="28" t="n">
+        <v>46252</v>
+      </c>
       <c r="K98" s="10" t="n"/>
     </row>
     <row r="99">
@@ -5044,7 +5064,7 @@
       </c>
       <c r="F99" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G99" s="12" t="inlineStr">
@@ -5058,7 +5078,9 @@
       <c r="I99" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J99" s="12" t="n"/>
+      <c r="J99" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K99" s="13" t="n"/>
     </row>
     <row r="100">
@@ -5089,7 +5111,7 @@
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
@@ -5103,7 +5125,9 @@
       <c r="I100" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J100" s="12" t="n"/>
+      <c r="J100" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K100" s="13" t="n"/>
     </row>
     <row r="101">
@@ -5134,7 +5158,7 @@
       </c>
       <c r="F101" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G101" s="12" t="inlineStr">
@@ -5148,7 +5172,9 @@
       <c r="I101" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J101" s="12" t="n"/>
+      <c r="J101" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K101" s="13" t="n"/>
     </row>
     <row r="102">
@@ -5179,7 +5205,7 @@
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
@@ -5193,7 +5219,9 @@
       <c r="I102" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J102" s="12" t="n"/>
+      <c r="J102" s="29" t="n">
+        <v>46246</v>
+      </c>
       <c r="K102" s="13" t="n"/>
     </row>
     <row r="103">
@@ -5224,7 +5252,7 @@
       </c>
       <c r="F103" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G103" s="12" t="inlineStr">
@@ -5238,8 +5266,14 @@
       <c r="I103" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J103" s="12" t="n"/>
-      <c r="K103" s="13" t="n"/>
+      <c r="J103" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K103" s="13" t="inlineStr">
+        <is>
+          <t>DatabaseReportSource wired to GET /api/reports (Validated-only, client-side filter); first real GPU fine-tune run 2026-08-17 (Colab T4), macro-F1 0.9520-&gt;0.9648, gate says promote. Not promoted yet -- pending adviser sign-off (would invalidate Sprint 5 threshold calibration, see 5.3.6). Merged to develop via PR #52 (75310ad), 2026-08-18.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
@@ -5363,7 +5397,7 @@
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
@@ -5377,8 +5411,14 @@
       <c r="I106" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J106" s="12" t="n"/>
-      <c r="K106" s="13" t="n"/>
+      <c r="J106" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K106" s="13" t="inlineStr">
+        <is>
+          <t>campaign_evolution.py (386 lines, pure module) + scripts/track_campaign_evolution.py (CLI) + 30 tests. Was stale here as In Progress; xlsx not updated when the code actually landed.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="12" t="inlineStr">
@@ -5455,7 +5495,7 @@
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
@@ -5469,8 +5509,14 @@
       <c r="I108" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J108" s="12" t="n"/>
-      <c r="K108" s="13" t="n"/>
+      <c r="J108" s="29" t="n">
+        <v>46250</v>
+      </c>
+      <c r="K108" s="13" t="inlineStr">
+        <is>
+          <t>Unknown Filter built: MessageFilter.UNKNOWN added to MessagesViewModel.kt, wired into MessagesScreen.kt's filter dropdown. compileDebugKotlin passes. Merged to develop via PR #46 (bc30c48).</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
@@ -5500,7 +5546,7 @@
       </c>
       <c r="F109" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G109" s="12" t="inlineStr">
@@ -5514,8 +5560,14 @@
       <c r="I109" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J109" s="12" t="n"/>
-      <c r="K109" s="13" t="n"/>
+      <c r="J109" s="29" t="n">
+        <v>46250</v>
+      </c>
+      <c r="K109" s="13" t="inlineStr">
+        <is>
+          <t>Now real end to end: new POST /api/ai/summarize backend proxy (JWT-guarded) forwards to the AI service's existing /summarize; new SummarizeApi.kt calls it from MessageDetailScreen.kt; AISummaryBottomSheet.kt renders the real summary and the fabricated 68%/92% confidence line was removed. Backend 167/167 tests pass. compileDebugKotlin passes. Merged to develop via PR #46 (bc30c48).</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
@@ -5545,7 +5597,7 @@
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
@@ -5559,8 +5611,14 @@
       <c r="I110" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J110" s="12" t="n"/>
-      <c r="K110" s="13" t="n"/>
+      <c r="J110" s="29" t="n">
+        <v>46250</v>
+      </c>
+      <c r="K110" s="13" t="inlineStr">
+        <is>
+          <t>Now synced both directions: new backend BlockedNumbersModule (GET/POST /api/blocked-numbers, DELETE /api/blocked-numbers/:sender); BlockedNumbersViewModel.kt reconciles device BlockedNumberContract against the backend on load and unblock hits both sides. Backend 167/167 tests pass. compileDebugKotlin passes. Merged to develop via PR #46 (bc30c48).</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="25.5" customHeight="1">
       <c r="A111" s="12" t="inlineStr">
@@ -5727,7 +5785,7 @@
       </c>
       <c r="F114" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G114" s="9" t="inlineStr">
@@ -5741,7 +5799,9 @@
       <c r="I114" s="25" t="n">
         <v>46282</v>
       </c>
-      <c r="J114" s="9" t="n"/>
+      <c r="J114" s="28" t="n">
+        <v>46252</v>
+      </c>
       <c r="K114" s="10" t="n"/>
     </row>
     <row r="115">
@@ -5772,7 +5832,7 @@
       </c>
       <c r="F115" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G115" s="12" t="inlineStr">
@@ -5786,8 +5846,14 @@
       <c r="I115" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J115" s="12" t="n"/>
-      <c r="K115" s="13" t="n"/>
+      <c r="J115" s="29" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K115" s="13" t="inlineStr">
+        <is>
+          <t>Covered across both tracks: reports.service.spec.ts (18 tests, report intake) + ai/tests/test_reports.py (31 tests, dataset append via DatabaseReportSource). Was stale here as Not Started.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="12" t="inlineStr">
@@ -5864,7 +5930,7 @@
       </c>
       <c r="F117" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G117" s="12" t="inlineStr">
@@ -5878,8 +5944,14 @@
       <c r="I117" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J117" s="12" t="n"/>
-      <c r="K117" s="13" t="n"/>
+      <c r="J117" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K117" s="13" t="inlineStr">
+        <is>
+          <t>Backend /retrain route + queue and ModelVersions registration built and verified live against real Docker Postgres + backend + AI service (scripts/round_trip.py, all 5 stages passed). ModelVersions given its first real row (2026-07-29 checkpoint, active). Unblocks 4.5.1. Merged to develop via PR #53 (72b78a8), 2026-08-18.</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="25.5" customHeight="1">
       <c r="A118" s="9" t="inlineStr">
@@ -5905,7 +5977,7 @@
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G118" s="9" t="inlineStr">
@@ -5919,7 +5991,9 @@
       <c r="I118" s="25" t="n">
         <v>46282</v>
       </c>
-      <c r="J118" s="9" t="n"/>
+      <c r="J118" s="28" t="n">
+        <v>46252</v>
+      </c>
       <c r="K118" s="10" t="n"/>
     </row>
     <row r="119">
@@ -5950,7 +6024,7 @@
       </c>
       <c r="F119" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G119" s="12" t="inlineStr">
@@ -5964,8 +6038,14 @@
       <c r="I119" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J119" s="12" t="n"/>
-      <c r="K119" s="13" t="n"/>
+      <c r="J119" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K119" s="13" t="inlineStr">
+        <is>
+          <t>Independently re-verified (not just Maxene write-up): round_trip.py re-run live against real Docker Postgres + backend + AI service, all 5 stages passed. Local env needed a migrate deploy and the real INTERNAL_API_KEY -- both environment gaps, not code bugs.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
@@ -5991,7 +6071,7 @@
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
@@ -6005,8 +6085,14 @@
       <c r="I120" s="26" t="n">
         <v>46282</v>
       </c>
-      <c r="J120" s="12" t="n"/>
-      <c r="K120" s="13" t="n"/>
+      <c r="J120" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K120" s="13" t="inlineStr">
+        <is>
+          <t>Retro held 2026-08-18. Went well: Build/Test/Demo all independently re-verified, not just taken on one contributor's word. Known limitation carried to Sprint 5/6, not a Sprint 4 blocker: mobile app has no deployed backend yet -- Alerts/Campaigns screens only work tethered to a laptop (adb reverse / 10.0.2.2). Real deployment is explicitly Sprint 6 scope.</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="25.5" customHeight="1">
       <c r="A121" s="6" t="inlineStr">
@@ -6290,7 +6376,7 @@
       </c>
       <c r="F127" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G127" s="12" t="inlineStr">
@@ -6304,8 +6390,14 @@
       <c r="I127" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="J127" s="12" t="n"/>
-      <c r="K127" s="13" t="n"/>
+      <c r="J127" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K127" s="13" t="inlineStr">
+        <is>
+          <t>ai/REFINEMENT_PLAN.md written -- refinement reuses Sprint 4 retraining pipeline unchanged; already executed once (4.3.5, 2026-08-17, promote verdict). Remaining work is the promotion decision itself, gated under 5.3.6. Merged via PR #54 (5b1ca27), 2026-08-18.</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="25.5" customHeight="1">
       <c r="A128" s="9" t="inlineStr">
@@ -6603,7 +6695,7 @@
       </c>
       <c r="F134" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G134" s="12" t="inlineStr">
@@ -6648,7 +6740,7 @@
       </c>
       <c r="F135" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G135" s="12" t="inlineStr">
@@ -6662,8 +6754,14 @@
       <c r="I135" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="J135" s="12" t="n"/>
-      <c r="K135" s="13" t="n"/>
+      <c r="J135" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K135" s="13" t="inlineStr">
+        <is>
+          <t>Measured via new scripts/analyze_indicator_coverage.py against every labeled Spam/Scam row. Scam zero-tag rate 48.6%-&gt;40.0% after adding Tagalog online-betting vocabulary + a phishing phrasing gap; Ham false-positive check &lt;0.1%. test_indicator_tags.py 17-&gt;20 tests. Merged via PR #54 (5b1ca27), 2026-08-18.</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="25.5" customHeight="1">
       <c r="A136" s="12" t="inlineStr">
@@ -6689,7 +6787,7 @@
       </c>
       <c r="F136" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G136" s="12" t="inlineStr">
@@ -6703,8 +6801,14 @@
       <c r="I136" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="J136" s="12" t="n"/>
-      <c r="K136" s="13" t="n"/>
+      <c r="J136" s="29" t="n">
+        <v>46254</v>
+      </c>
+      <c r="K136" s="13" t="inlineStr">
+        <is>
+          <t>Two Explore passes audited the full mobile source tree; fixed a real SmsReceiver crash (empty message array from a failed multipart PDU), blank-sender bugs (normalizeAddress/getInitialsFromSender), a negative-clock-skew display bug (getRelativeTime), missing error handling + load races in Home/Messages/MessageDetail ViewModels, a phone-number validation rewrite, and an IME-scroll fix across 3 onboarding screens. Also caught and fixed live mid-session: an EMUI floating-window gesture crash (MainActivity now declares resizeableActivity=false + configChanges). All fixes live-verified on Gio's physical device except SmsReceiver's empty-PDU guard (code-review only -- not injectable on real hardware). Merged via PR #59 (8e1567d), 2026-08-20.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
@@ -6730,7 +6834,7 @@
       </c>
       <c r="F137" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G137" s="12" t="inlineStr">
@@ -6744,8 +6848,14 @@
       <c r="I137" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="J137" s="12" t="n"/>
-      <c r="K137" s="13" t="n"/>
+      <c r="J137" s="29" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K137" s="13" t="inlineStr">
+        <is>
+          <t>Ran the real onboarding-through-main-app flow live on an emulator. Real bugs found and fixed: Terms/Allow-Access screens built but never wired into NavGraph; phone numbers stored without +63 prefix; disabled-button state missing; bottom-nav badge hardcoded/inconsistent (now bound to real AlertsViewModel data); dead back button; avatar-initials lag. Redesigned profile screen (staggered animation, spring bounce) + app-wide screen transitions + tab cross-fade. ktlint/detekt/build all clean.</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="25.5" customHeight="1">
       <c r="A138" s="12" t="inlineStr">
@@ -6861,7 +6971,7 @@
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G140" s="9" t="inlineStr">
@@ -6996,7 +7106,7 @@
       </c>
       <c r="F143" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G143" s="12" t="inlineStr">
@@ -7010,8 +7120,14 @@
       <c r="I143" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="J143" s="12" t="n"/>
-      <c r="K143" s="13" t="n"/>
+      <c r="J143" s="29" t="n">
+        <v>46254</v>
+      </c>
+      <c r="K143" s="13" t="inlineStr">
+        <is>
+          <t>Scoped to static SDK_INT review (all 4 version-gated branches confirmed correct by reading the guarded code) + live device testing, since no Android 11+ emulator with working telephony/System UI was available this session. Live verification happened on Android 10/API 29 (Huawei VOG-L29) -- one version below the Android 11+ this task names. Accepted given minSdk 26/targetSdk 35 covers the full range and real device testing caught a genuine EMUI crash an emulator likely wouldn't have. Merged via PR #59 (8e1567d), 2026-08-20.</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="25.5" customHeight="1">
       <c r="A144" s="9" t="inlineStr">
@@ -7164,7 +7280,7 @@
       </c>
       <c r="F147" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G147" s="6" t="inlineStr">
@@ -7905,7 +8021,7 @@
       </c>
       <c r="F164" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G164" s="9" t="inlineStr">
@@ -8167,7 +8283,7 @@
       </c>
       <c r="F170" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G170" s="12" t="inlineStr">
@@ -8182,7 +8298,11 @@
         <v>46324</v>
       </c>
       <c r="J170" s="12" t="n"/>
-      <c r="K170" s="13" t="n"/>
+      <c r="K170" s="13" t="inlineStr">
+        <is>
+          <t>Maxene, early prep ahead of Sprint 6 (both commits label it 'prep', not the final deliverable). create_holdout_set.py carved a permanent 20% held-out split (3,236 rows, grouped, seed 20260618). evaluate_holdout.py scored the currently-deployed checkpoint at macro-F1 0.95, but the holdout manifest itself caveats this isn't a clean test -- that model was trained before the split existed. The real 6.4.6 result needs the first model trained after 2026-08-18. Merged via PR #56/#58, 2026-08-20.</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="25.5" customHeight="1">
       <c r="A171" s="9" t="inlineStr">

</xml_diff>